<commit_message>
Placera KIM 1 och KIM 3 bredvid varandra
</commit_message>
<xml_diff>
--- a/AppLinks.xlsx
+++ b/AppLinks.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appar" sheetId="1" r:id="R514f02e3f6174184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appar" sheetId="1" r:id="Rdff51e18df8d497b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,66 +17,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Länk</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Standardiserad ergonomibedömning för operatörsarbete. Beräknar riskpoäng, visualiserar belastning och ger tydligt underlag för åtgärder.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://mrmartinpet.github.io/ErgonomicAnalysis/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Frekvensanalys</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visualiserar hur tid och aktiviteter fördelas över roller eller processer. Synliggör obalanser, överbelastning och förbättringspotential.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://mrmartinpet.github.io/Frekvensanalys/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">20CycleCheck</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Digitalt stöd för 20 Cycle Check och processobservation. Fångar variation, avvikelser och standardefterlevnad direkt vid processen.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://mrmartinpet.github.io/20CycleCheck/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">StepTimer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Realtidsmätning av cykeltid per processteg. Skapar snabb överblick över flaskhalsar, variation och taktavvikelse.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://mrmartinpet.github.io/steptimer/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Funktionsplaneraren</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Visualiserar ansvar och arbetsbelastning för indirekta funktioner. Gör det enklare att fördela uppgifter och säkra rätt fokus.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://mrmartinpet.github.io/Funktionsplaneraren/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Tolkkalibrering</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Digital app för kalibrering av håltolkar. Registrerar mätvärden, beräknar största avvikelse mot ±0,02 mm och ger direkt godkänd eller underkänd.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://mrmartinpet.github.io/Tolkkalibrering/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Flagg-generator</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Genererar och skriver ut pallflaggor för verktygspallar. Standardiserad märkning för tydlig identifiering och spårbarhet i produktionen.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://mrmartinpet.github.io/Flagg-generator/</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -314,98 +254,98 @@
       <x:c r="A2" t="str">
         <x:v>Ergonomianalys KIM 1</x:v>
       </x:c>
-      <x:c r="B2" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C2" t="s">
-        <x:v>4</x:v>
+      <x:c r="B2" t="str">
+        <x:v>Standardiserad ergonomibedömning för operatörsarbete. Beräknar riskpoäng, visualiserar belastning och ger tydligt underlag för åtgärder.</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>https://mrmartinpet.github.io/ErgonomicAnalysis/</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B3" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C3" t="s">
-        <x:v>7</x:v>
+      <x:c r="A3" t="str">
+        <x:v>Ergonomianalys KIM 3</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Digital riskbedömning av repetitivt arbete enligt KIM III. Beräknar riskpoäng och skapar en komplett A4-rapport.</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>https://mrmartinpet.github.io/KIM3/</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B4" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C4" s="2" t="s">
-        <x:v>10</x:v>
+      <x:c r="A4" t="str">
+        <x:v>Frekvensanalys</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Visualiserar hur tid och aktiviteter fördelas över roller eller processer. Synliggör obalanser, överbelastning och förbättringspotential.</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>https://mrmartinpet.github.io/Frekvensanalys/</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B5" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C5" t="s">
-        <x:v>13</x:v>
+      <x:c r="A5" t="str">
+        <x:v>20CycleCheck</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Digitalt stöd för 20 Cycle Check och processobservation. Fångar variation, avvikelser och standardefterlevnad direkt vid processen.</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>https://mrmartinpet.github.io/20CycleCheck/</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B6" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C6" t="s">
-        <x:v>16</x:v>
+      <x:c r="A6" t="str">
+        <x:v>StepTimer</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Realtidsmätning av cykeltid per processteg. Skapar snabb överblick över flaskhalsar, variation och taktavvikelse.</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>https://mrmartinpet.github.io/steptimer/</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B7" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C7" s="2" t="s">
-        <x:v>19</x:v>
+      <x:c r="A7" t="str">
+        <x:v>Funktionsplaneraren</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Visualiserar ansvar och arbetsbelastning för indirekta funktioner. Gör det enklare att fördela uppgifter och säkra rätt fokus.</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>https://mrmartinpet.github.io/Funktionsplaneraren/</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B8" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="C8" t="s">
-        <x:v>22</x:v>
+      <x:c r="A8" t="str">
+        <x:v>Tolkkalibrering</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Digital app för kalibrering av håltolkar. Registrerar mätvärden, beräknar största avvikelse mot ±0,02 mm och ger direkt godkänd eller underkänd.</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>https://mrmartinpet.github.io/Tolkkalibrering/</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Ergonomianalys KIM 3</x:v>
+        <x:v>Flagg-generator</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Digital riskbedömning av repetitivt arbete enligt KIM III. Beräknar riskpoäng och skapar en komplett A4-rapport.</x:v>
+        <x:v>Genererar och skriver ut pallflaggor för verktygspallar. Standardiserad märkning för tydlig identifiering och spårbarhet i produktionen.</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>https://mrmartinpet.github.io/KIM3/</x:v>
+        <x:v>https://mrmartinpet.github.io/Flagg-generator/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R2a56a7d5e4f24164"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="R3610d91b6580478f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R032ed7be85214799"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="R62d8d61cf8be4d59"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R656569639fbe4db3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra47f00ff4833407a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Samordna beskrivningarna för KIM 1 och KIM 3
</commit_message>
<xml_diff>
--- a/AppLinks.xlsx
+++ b/AppLinks.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appar" sheetId="1" r:id="Rdff51e18df8d497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Appar" sheetId="1" r:id="R7495d63907414267"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -255,7 +255,7 @@
         <x:v>Ergonomianalys KIM 1</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Standardiserad ergonomibedömning för operatörsarbete. Beräknar riskpoäng, visualiserar belastning och ger tydligt underlag för åtgärder.</x:v>
+        <x:v>Digital riskbedömning av lyft och bärande enligt KIM I. Beräknar riskpoäng och skapar en komplett A4-rapport.</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>https://mrmartinpet.github.io/ErgonomicAnalysis/</x:v>
@@ -340,12 +340,12 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R032ed7be85214799"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="R62d8d61cf8be4d59"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="R47a90226f10b4031"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="Rcb52aa34a87049cc"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra47f00ff4833407a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba9b67d7387949db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>